<commit_message>
fix(pptx): merged table cells read with their spans
A cell's gridSpan and rowSpan are its colSpan and rowSpan, and the positions it covers (hMerge, vMerge) are no cells of their own: they were read as empty cells, and the merge was lost.
</commit_message>
<xml_diff>
--- a/test/generator/baseline/gen.pptx.to.xlsx.xlsx
+++ b/test/generator/baseline/gen.pptx.to.xlsx.xlsx
@@ -513,6 +513,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
 </worksheet>
 </file>
 
@@ -542,7 +545,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
@@ -1308,6 +1311,21 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+  </mergeCells>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(pdf): keepHeadersAndFootersInPages keeps running headers and footers in their pages
A tagged PDF marks its running headers and footers as artifacts, and they are read into auxiliary,
where writers that lay out no pages (text, Markdown, HTML, EPUB, slides) leave them out. With
pdfParserConfig.keepHeadersAndFootersInPages each page keeps its own in its content, the header before
the page's text and the footer after it, placed before the page's pictures are, for a page-faithful
result such as a slide per page. ignoreHeadersAndFooters still drops them. Baselines carry the new key
and the automatic chart titles of the last commit.
</commit_message>
<xml_diff>
--- a/test/generator/baseline/gen.pptx.to.xlsx.xlsx
+++ b/test/generator/baseline/gen.pptx.to.xlsx.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Tables 4" sheetId="4" r:id="rId4"/>
     <sheet name="Tables 5" sheetId="5" r:id="rId5"/>
     <sheet name="Tables 6" sheetId="6" r:id="rId6"/>
-    <sheet name="Charts Chart" sheetId="7" r:id="rId7"/>
+    <sheet name="Chart Title" sheetId="7" r:id="rId7"/>
     <sheet name="Text" sheetId="8" r:id="rId8"/>
     <sheet name="Notes" sheetId="9" r:id="rId9"/>
   </sheets>
@@ -1348,51 +1348,40 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chart Title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
         <is>
           <t xml:space="preserve">Series 1</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t xml:space="preserve">Series 2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t xml:space="preserve">Series 3</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Category 1</t>
-        </is>
-      </c>
-      <c r="B2" s="3">
-        <v>4.3</v>
-      </c>
-      <c r="C2" s="3">
-        <v>2.4</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Category 2</t>
+          <t xml:space="preserve">Category 1</t>
         </is>
       </c>
       <c r="B3" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.4000000000000004</t>
-        </is>
+        <v>4.3</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2.4</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -1401,36 +1390,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Category 3</t>
+          <t xml:space="preserve">Category 2</t>
         </is>
       </c>
       <c r="B4" s="3">
-        <v>3.5</v>
-      </c>
-      <c r="C4" s="3">
-        <v>1.8</v>
+        <v>2.5</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.4000000000000004</t>
+        </is>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Category 3</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Category 4</t>
         </is>
       </c>
-      <c r="B5" s="3">
+      <c r="B6" s="3">
         <v>4.5</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C6" s="3">
         <v>2.8</v>
       </c>
-      <c r="D5">
+      <c r="D6">
         <v>5</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
 </worksheet>
 </file>
 

</xml_diff>